<commit_message>
Agregar escritura Supabase para CRM
</commit_message>
<xml_diff>
--- a/data/crm_restaurantes_estado.xlsx
+++ b/data/crm_restaurantes_estado.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1103,6 +1103,51 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Kechua+Vitacura/@-33.3817562,-70.57943,17z/data=!3m1!4b1!4m6!3m5!1s0x9662c91a55258adf:0x8b4d8fd1119ebaae!8m2!3d-33.3817562!4d-70.57943!16s%2Fg%2F11sj5dh_jm?authuser=0&amp;hl=es-419&amp;entry=ttu&amp;g_ep=EgoyMDI2MDUxNy4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-05-22 15:41:32</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Llamada</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Llamada iniciada desde CRM</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>